<commit_message>
started tagging existing decklists with archetype tags, intend to train a ml to determine archetypes in future.  created function in decks.py to format data for ml code, deck_images.py for visualization
</commit_message>
<xml_diff>
--- a/input/xlsx/90.xlsx
+++ b/input/xlsx/90.xlsx
@@ -4,20 +4,21 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Draft" sheetId="1" r:id="rId1"/>
     <sheet name="Play" sheetId="2" r:id="rId2"/>
     <sheet name="Results" sheetId="3" r:id="rId3"/>
     <sheet name="Date" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="196">
   <si>
     <t>Nenni</t>
   </si>
@@ -602,6 +603,9 @@
   </si>
   <si>
     <t>5.0</t>
+  </si>
+  <si>
+    <t>bao savant upheaval</t>
   </si>
 </sst>
 </file>
@@ -2892,4 +2896,19 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>